<commit_message>
Complete phase 3 package workspace
</commit_message>
<xml_diff>
--- a/backend_tracker_solo_professional.xlsx
+++ b/backend_tracker_solo_professional.xlsx
@@ -427,7 +427,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:O20"/>
   <sheetFormatPr defaultRowHeight="22"/>
   <cols>
@@ -990,11 +990,11 @@
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J8" s="22">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K8" s="15" t="inlineStr">
         <is>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="N8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uu tien data model ro rang truoc khi lam UI</t>
+          <t>Done 2026-04-16: package CRUD, assign, archive/restore, and /package-catalog split completed.</t>
         </is>
       </c>
     </row>
@@ -1061,11 +1061,11 @@
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J9" s="22">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K9" s="14" t="inlineStr">
         <is>
@@ -1084,12 +1084,12 @@
       </c>
       <c r="N9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Day la logic nghiep vu can test ky</t>
+          <t>Done 2026-04-16: usage aggregation, timeline, export CSV, and filters completed.</t>
         </is>
       </c>
     </row>
@@ -1132,11 +1132,11 @@
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J10" s="22">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K10" s="14" t="inlineStr">
         <is>
@@ -1155,12 +1155,12 @@
       </c>
       <c r="N10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Neu thieu thoi gian, block tu dong co the de phase sau</t>
+          <t>Done 2026-04-16: quota tracking, alerts, and assignment lifecycle detail completed.</t>
         </is>
       </c>
     </row>
@@ -1203,11 +1203,11 @@
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J11" s="22">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="N11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dong phase khi so lieu usage da dang tin</t>
+          <t>Done 2026-04-16: audit history and NOC-friendly advanced UX finalized.</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="22"/>
   <cols>
@@ -2083,17 +2083,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lam nghiep vu tao gia tri som</t>
+          <t>Lam nghiep vu package/usage va hoan thien UX cho NOC</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Package CRUD; quota logic; user usage; usage aggregation; alert co ban</t>
+          <t>Package CRUD; quota logic; user usage; usage aggregation; alert co ban; audit/export; lifecycle detail</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tinh va hien thi duoc usage theo user, quota hoat dong dung</t>
+          <t>Tinh va hien thi duoc usage theo user, quota hoat dong dung, audit/export/lifecycle detail san sang</t>
         </is>
       </c>
       <c r="H5" s="17" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tap trung dung du lieu truoc khi polish UI</t>
+          <t>Completed 2026-04-16: /dashboard is monitoring-only; /package-catalog handles package operations and advanced reporting.</t>
         </is>
       </c>
     </row>

</xml_diff>